<commit_message>
`Change supply and create api download file sample import tool`
</commit_message>
<xml_diff>
--- a/src/main/resources/static/Sample_Excel_Import_Tool.xlsx
+++ b/src/main/resources/static/Sample_Excel_Import_Tool.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hieux\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hieux\Desktop\Projects\src\main\resources\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0713145E-10D9-4230-A00F-14023699BCF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2FDEFE7-9EBC-4406-85CA-E2ADF7F77D89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{69C10241-C50D-4A10-BA91-0773532975B3}"/>
   </bookViews>
@@ -378,9 +378,6 @@
     <t>Bao gồm các nhóm loại công cụ dụng cụ đã được xác định trong hệ thống. Người dùng sẽ chọn  công cụ dụng cụ đã được xác định từ danh sách công cụ dụng cụ.</t>
   </si>
   <si>
-    <t>Nhà cung cấp dùng để xác định thông tin của nhà cung cấp. Người dùng nên ghi rõ thông tin về nhà cung cấp (Bao gồm: Tên nhà cung cấp, địa chỉ, mã số thuế,... (nếu có))</t>
-  </si>
-  <si>
     <t>Số Quyết định là số hiệu của quyết định do đơn vị cấp phát (trang cấp) công cụ dụng cụ.</t>
   </si>
   <si>
@@ -461,6 +458,9 @@
   <si>
     <t>Nguồn hình thành là các nguồn vốn hoặc tài chính được sử dụng để mua sắm, xây dựng hoặc tạo ra công cụ dụng cụ cho đơn vị. Từ đó tính ra giá trị nguyên giá ghi theo sổ kế toán. Ví dụ:
 Ngân sách Huyện tự chủ;Ngân sách Xã;Nguồn tài trợ - viện trợ</t>
+  </si>
+  <si>
+    <t>Nhà cung cấp dùng để xác định thông tin của nhà cung cấp. Danh sách nhà cung cấp đã được xác định trong hệ thống.</t>
   </si>
 </sst>
 </file>
@@ -604,14 +604,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -619,7 +628,7 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -633,17 +642,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -982,177 +980,177 @@
   <dimension ref="A1:Z14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" style="12" customWidth="1"/>
-    <col min="2" max="2" width="25.7109375" style="12" customWidth="1"/>
-    <col min="3" max="3" width="26.85546875" style="12" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" style="12" customWidth="1"/>
-    <col min="5" max="6" width="20.42578125" style="12" customWidth="1"/>
-    <col min="7" max="7" width="20.85546875" style="12" customWidth="1"/>
-    <col min="8" max="8" width="31.85546875" style="12" customWidth="1"/>
-    <col min="9" max="9" width="15.5703125" style="12" customWidth="1"/>
-    <col min="10" max="10" width="15.7109375" style="12" customWidth="1"/>
-    <col min="11" max="11" width="18.42578125" style="12" customWidth="1"/>
-    <col min="12" max="12" width="18.85546875" style="12" customWidth="1"/>
-    <col min="13" max="13" width="16.28515625" style="12" customWidth="1"/>
-    <col min="14" max="14" width="18.140625" style="12" customWidth="1"/>
-    <col min="15" max="15" width="18" style="12" customWidth="1"/>
-    <col min="16" max="16" width="20.85546875" style="12" customWidth="1"/>
-    <col min="17" max="17" width="19.140625" style="12" customWidth="1"/>
-    <col min="18" max="18" width="24.7109375" style="12" customWidth="1"/>
-    <col min="19" max="19" width="17.28515625" style="12" customWidth="1"/>
-    <col min="20" max="20" width="18" style="12" customWidth="1"/>
-    <col min="21" max="21" width="18.5703125" style="12" customWidth="1"/>
-    <col min="22" max="22" width="18.28515625" style="12" customWidth="1"/>
-    <col min="23" max="23" width="14.85546875" style="12" customWidth="1"/>
-    <col min="24" max="24" width="9.140625" style="12"/>
-    <col min="25" max="25" width="14.140625" style="12" customWidth="1"/>
-    <col min="26" max="26" width="13.28515625" style="12" customWidth="1"/>
-    <col min="27" max="16384" width="9.140625" style="12"/>
+    <col min="1" max="1" width="24.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="29.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" style="1" customWidth="1"/>
+    <col min="5" max="6" width="20.42578125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.85546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="31.85546875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="15.7109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="18.42578125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="18.85546875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="16.28515625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="18.140625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="18" style="1" customWidth="1"/>
+    <col min="16" max="16" width="20.85546875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="19.140625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="24.7109375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="17.28515625" style="1" customWidth="1"/>
+    <col min="20" max="20" width="18" style="1" customWidth="1"/>
+    <col min="21" max="21" width="18.5703125" style="1" customWidth="1"/>
+    <col min="22" max="22" width="18.28515625" style="1" customWidth="1"/>
+    <col min="23" max="23" width="14.85546875" style="1" customWidth="1"/>
+    <col min="24" max="24" width="9.140625" style="1"/>
+    <col min="25" max="25" width="14.140625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="13.28515625" style="1" customWidth="1"/>
+    <col min="27" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="8" t="s">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
-      <c r="P1" s="9" t="s">
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="Q1" s="9"/>
-      <c r="R1" s="9"/>
-      <c r="S1" s="10" t="s">
+      <c r="Q1" s="12"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="T1" s="10"/>
-      <c r="U1" s="10"/>
-      <c r="V1" s="10"/>
-      <c r="W1" s="10"/>
-      <c r="X1" s="10"/>
-      <c r="Y1" s="10"/>
-      <c r="Z1" s="10"/>
+      <c r="T1" s="13"/>
+      <c r="U1" s="13"/>
+      <c r="V1" s="13"/>
+      <c r="W1" s="13"/>
+      <c r="X1" s="13"/>
+      <c r="Y1" s="13"/>
+      <c r="Z1" s="13"/>
     </row>
     <row r="2" spans="1:26" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="P2" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="5" t="s">
+      <c r="Q2" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="R2" s="5" t="s">
+      <c r="R2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="S2" s="11" t="s">
+      <c r="S2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="T2" s="11"/>
-      <c r="U2" s="11"/>
-      <c r="V2" s="11"/>
-      <c r="W2" s="11"/>
-      <c r="X2" s="11"/>
-      <c r="Y2" s="11"/>
-      <c r="Z2" s="11"/>
+      <c r="T2" s="4"/>
+      <c r="U2" s="4"/>
+      <c r="V2" s="4"/>
+      <c r="W2" s="4"/>
+      <c r="X2" s="4"/>
+      <c r="Y2" s="4"/>
+      <c r="Z2" s="4"/>
     </row>
     <row r="3" spans="1:26" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="5"/>
-      <c r="R3" s="5"/>
-      <c r="S3" s="6" t="s">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="8"/>
+      <c r="Q3" s="8"/>
+      <c r="R3" s="8"/>
+      <c r="S3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="T3" s="6" t="s">
+      <c r="T3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="U3" s="6" t="s">
+      <c r="U3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="V3" s="6" t="s">
+      <c r="V3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="W3" s="6" t="s">
+      <c r="W3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="X3" s="6" t="s">
+      <c r="X3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="Y3" s="6" t="s">
+      <c r="Y3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="Z3" s="6" t="s">
+      <c r="Z3" s="3" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1164,116 +1162,126 @@
         <v>31</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="H4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="I4" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="M4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="N4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="O4" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="O4" s="2" t="s">
+      <c r="P4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="P4" s="2" t="s">
+      <c r="Q4" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="Q4" s="2" t="s">
+      <c r="R4" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="S4" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="S4" s="2" t="s">
-        <v>48</v>
       </c>
       <c r="T4" s="2" t="s">
         <v>23</v>
       </c>
       <c r="U4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="V4" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="V4" s="2" t="s">
+      <c r="W4" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="W4" s="2" t="s">
-        <v>51</v>
       </c>
       <c r="X4" s="2"/>
       <c r="Y4" s="2"/>
       <c r="Z4" s="2"/>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
+      <c r="A7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A8" s="14"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A9" s="14"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A10" s="14"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A11" s="14"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A12" s="14"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A13" s="14"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A14" s="14"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="I1:O1"/>
+    <mergeCell ref="P1:R1"/>
+    <mergeCell ref="S1:Z1"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:F3"/>
     <mergeCell ref="S2:Z2"/>
     <mergeCell ref="A7:C14"/>
     <mergeCell ref="M2:M3"/>
@@ -1288,16 +1296,6 @@
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="K2:K3"/>
     <mergeCell ref="L2:L3"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="I1:O1"/>
-    <mergeCell ref="P1:R1"/>
-    <mergeCell ref="S1:Z1"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="F2:F3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1305,7 +1303,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01287988-01F9-4CC5-B1A4-5B062B8BCC20}">
-  <dimension ref="A1:Z4"/>
+  <dimension ref="A1:Z3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" style="1" customWidth="1"/>
@@ -1326,168 +1324,153 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="8" t="s">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
-      <c r="P1" s="9" t="s">
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="Q1" s="9"/>
-      <c r="R1" s="9"/>
-      <c r="S1" s="10" t="s">
+      <c r="Q1" s="12"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="T1" s="10"/>
-      <c r="U1" s="10"/>
-      <c r="V1" s="10"/>
-      <c r="W1" s="10"/>
-      <c r="X1" s="10"/>
-      <c r="Y1" s="10"/>
-      <c r="Z1" s="10"/>
+      <c r="T1" s="13"/>
+      <c r="U1" s="13"/>
+      <c r="V1" s="13"/>
+      <c r="W1" s="13"/>
+      <c r="X1" s="13"/>
+      <c r="Y1" s="13"/>
+      <c r="Z1" s="13"/>
     </row>
     <row r="2" spans="1:26" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="P2" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="5" t="s">
+      <c r="Q2" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="R2" s="5" t="s">
+      <c r="R2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="S2" s="11" t="s">
+      <c r="S2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="T2" s="11"/>
-      <c r="U2" s="11"/>
-      <c r="V2" s="11"/>
-      <c r="W2" s="11"/>
-      <c r="X2" s="11"/>
-      <c r="Y2" s="11"/>
-      <c r="Z2" s="11"/>
+      <c r="T2" s="4"/>
+      <c r="U2" s="4"/>
+      <c r="V2" s="4"/>
+      <c r="W2" s="4"/>
+      <c r="X2" s="4"/>
+      <c r="Y2" s="4"/>
+      <c r="Z2" s="4"/>
     </row>
     <row r="3" spans="1:26" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="5"/>
-      <c r="R3" s="5"/>
-      <c r="S3" s="6" t="s">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="8"/>
+      <c r="Q3" s="8"/>
+      <c r="R3" s="8"/>
+      <c r="S3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="T3" s="6" t="s">
+      <c r="T3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="U3" s="6" t="s">
+      <c r="U3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="V3" s="6" t="s">
+      <c r="V3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="W3" s="6" t="s">
+      <c r="W3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="X3" s="6" t="s">
+      <c r="X3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="Y3" s="6" t="s">
+      <c r="Y3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="Z3" s="6" t="s">
+      <c r="Z3" s="3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="U4" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="R2:R3"/>
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
-    <mergeCell ref="P2:P3"/>
-    <mergeCell ref="Q2:Q3"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:J3"/>
     <mergeCell ref="K2:K3"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="I1:O1"/>
@@ -1499,6 +1482,18 @@
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="R2:R3"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="Q2:Q3"/>
   </mergeCells>
   <dataValidations count="9">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Tình trạng sử dụng của công cụ dụng cụ: Còn sử dụng được và Không sử dụng được" sqref="N4:N2003" xr:uid="{D7D8503B-1533-4BDA-9D09-20E03F393295}">

</xml_diff>

<commit_message>
Create api download template import tool
</commit_message>
<xml_diff>
--- a/src/main/resources/static/Sample_Excel_Import_Tool.xlsx
+++ b/src/main/resources/static/Sample_Excel_Import_Tool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hieux\Desktop\Projects\src\main\resources\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A98F322B-D91D-438C-97CF-AB224F8DCA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F4B9E5-FA6C-4A76-AB62-B973D400952E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{69C10241-C50D-4A10-BA91-0773532975B3}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{69C10241-C50D-4A10-BA91-0773532975B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Huongdannhapthongtin" sheetId="2" r:id="rId1"/>
@@ -375,9 +375,6 @@
     <t>Tên công cụ dụng cụ được sử dụng để phân biệt các công cụ dụng cụ. Người dùng nên đặt tên tài sản theo cú pháp quy ước để thuận tiện cho việc tra cứu, tìm kiếm.</t>
   </si>
   <si>
-    <t>Bao gồm các nhóm loại công cụ dụng cụ đã được xác định trong hệ thống. Người dùng sẽ chọn  công cụ dụng cụ đã được xác định từ danh sách công cụ dụng cụ.</t>
-  </si>
-  <si>
     <t>Số Quyết định là số hiệu của quyết định do đơn vị cấp phát (trang cấp) công cụ dụng cụ.</t>
   </si>
   <si>
@@ -461,6 +458,10 @@
   </si>
   <si>
     <t>Nhà cung cấp dùng để xác định thông tin của nhà cung cấp. Danh sách nhà cung cấp đã được xác định trong hệ thống.</t>
+  </si>
+  <si>
+    <t>Bao gồm các nhóm loại công cụ dụng cụ đã được xác định trong hệ thống. Người dùng sẽ chọn  công cụ dụng cụ đã được xác định từ danh sách công cụ dụng cụ.
+Người dùng có thể mở sheet "ToolCategoriesView" để xem danh sách danh mục công cụ dụng cụ tương ứng.</t>
   </si>
 </sst>
 </file>
@@ -667,7 +668,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -676,6 +677,21 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -688,24 +704,9 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -730,6 +731,13 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1096,40 +1104,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="5" t="s">
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
-      <c r="N1" s="5"/>
-      <c r="O1" s="5"/>
-      <c r="P1" s="6" t="s">
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="Q1" s="6"/>
-      <c r="R1" s="6"/>
-      <c r="S1" s="7" t="s">
+      <c r="Q1" s="11"/>
+      <c r="R1" s="11"/>
+      <c r="S1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="T1" s="7"/>
-      <c r="U1" s="7"/>
-      <c r="V1" s="7"/>
-      <c r="W1" s="7"/>
-      <c r="X1" s="7"/>
-      <c r="Y1" s="7"/>
-      <c r="Z1" s="7"/>
+      <c r="T1" s="12"/>
+      <c r="U1" s="12"/>
+      <c r="V1" s="12"/>
+      <c r="W1" s="12"/>
+      <c r="X1" s="12"/>
+      <c r="Y1" s="12"/>
+      <c r="Z1" s="12"/>
     </row>
     <row r="2" spans="1:26" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
@@ -1156,46 +1164,46 @@
       <c r="H2" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="12" t="s">
+      <c r="J2" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="12" t="s">
+      <c r="K2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="12" t="s">
+      <c r="L2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="12" t="s">
+      <c r="M2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="12" t="s">
+      <c r="N2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="12" t="s">
+      <c r="O2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="P2" s="13" t="s">
+      <c r="P2" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="13" t="s">
+      <c r="Q2" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="R2" s="13" t="s">
+      <c r="R2" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="S2" s="9" t="s">
+      <c r="S2" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="T2" s="9"/>
-      <c r="U2" s="9"/>
-      <c r="V2" s="9"/>
-      <c r="W2" s="9"/>
-      <c r="X2" s="9"/>
-      <c r="Y2" s="9"/>
-      <c r="Z2" s="9"/>
+      <c r="T2" s="13"/>
+      <c r="U2" s="13"/>
+      <c r="V2" s="13"/>
+      <c r="W2" s="13"/>
+      <c r="X2" s="13"/>
+      <c r="Y2" s="13"/>
+      <c r="Z2" s="13"/>
     </row>
     <row r="3" spans="1:26" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
@@ -1206,16 +1214,16 @@
       <c r="F3" s="8"/>
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="12"/>
-      <c r="O3" s="12"/>
-      <c r="P3" s="13"/>
-      <c r="Q3" s="13"/>
-      <c r="R3" s="13"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
       <c r="S3" s="3" t="s">
         <v>22</v>
       </c>
@@ -1241,135 +1249,124 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="153" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" ht="179.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="H4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="I4" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="M4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="N4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="O4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="O4" s="2" t="s">
+      <c r="P4" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="P4" s="2" t="s">
+      <c r="Q4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="Q4" s="2" t="s">
+      <c r="R4" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="S4" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="S4" s="2" t="s">
-        <v>47</v>
       </c>
       <c r="T4" s="2" t="s">
         <v>23</v>
       </c>
       <c r="U4" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="V4" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="V4" s="2" t="s">
+      <c r="W4" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="W4" s="2" t="s">
-        <v>50</v>
       </c>
       <c r="X4" s="2"/>
       <c r="Y4" s="2"/>
       <c r="Z4" s="2"/>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
+      <c r="A7" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A8" s="11"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A9" s="11"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A10" s="11"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
+      <c r="A13" s="5"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A7:C14"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
-    <mergeCell ref="P2:P3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="L2:L3"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="I1:O1"/>
     <mergeCell ref="P1:R1"/>
@@ -1383,6 +1380,17 @@
     <mergeCell ref="S2:Z2"/>
     <mergeCell ref="Q2:Q3"/>
     <mergeCell ref="R2:R3"/>
+    <mergeCell ref="A7:C14"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="L2:L3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1390,14 +1398,22 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01287988-01F9-4CC5-B1A4-5B062B8BCC20}">
-  <dimension ref="A1:Z3"/>
+  <dimension ref="A1:Z4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" style="1" customWidth="1"/>
-    <col min="2" max="3" width="11.5703125" style="1" customWidth="1"/>
-    <col min="4" max="6" width="9.140625" style="1"/>
-    <col min="7" max="7" width="13.28515625" style="1" customWidth="1"/>
-    <col min="8" max="13" width="9.140625" style="1"/>
+    <col min="1" max="1" width="27.85546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18" style="1" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="15" style="1" customWidth="1"/>
+    <col min="10" max="10" width="17.85546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="19" style="1" customWidth="1"/>
+    <col min="12" max="12" width="18.140625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="19.28515625" style="1" customWidth="1"/>
     <col min="14" max="14" width="18" style="1" customWidth="1"/>
     <col min="15" max="18" width="9.140625" style="1"/>
     <col min="19" max="19" width="11.85546875" style="1" customWidth="1"/>
@@ -1420,31 +1436,31 @@
       <c r="E1" s="17"/>
       <c r="F1" s="17"/>
       <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="19" t="s">
+      <c r="H1" s="18"/>
+      <c r="I1" s="19" t="s">
         <v>1</v>
       </c>
+      <c r="J1" s="20"/>
       <c r="K1" s="20"/>
       <c r="L1" s="20"/>
       <c r="M1" s="20"/>
       <c r="N1" s="20"/>
       <c r="O1" s="21"/>
-      <c r="P1" s="6" t="s">
+      <c r="P1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="Q1" s="6"/>
-      <c r="R1" s="6"/>
-      <c r="S1" s="7" t="s">
+      <c r="Q1" s="11"/>
+      <c r="R1" s="11"/>
+      <c r="S1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="T1" s="7"/>
-      <c r="U1" s="7"/>
-      <c r="V1" s="7"/>
-      <c r="W1" s="7"/>
-      <c r="X1" s="7"/>
-      <c r="Y1" s="7"/>
-      <c r="Z1" s="7"/>
+      <c r="T1" s="12"/>
+      <c r="U1" s="12"/>
+      <c r="V1" s="12"/>
+      <c r="W1" s="12"/>
+      <c r="X1" s="12"/>
+      <c r="Y1" s="12"/>
+      <c r="Z1" s="12"/>
     </row>
     <row r="2" spans="1:26" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
@@ -1453,84 +1469,84 @@
       <c r="B2" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="J2" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="K2" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="L2" s="12" t="s">
+      <c r="L2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="12" t="s">
+      <c r="M2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="12" t="s">
+      <c r="N2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="12" t="s">
+      <c r="O2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="P2" s="13" t="s">
+      <c r="P2" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="13" t="s">
+      <c r="Q2" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="R2" s="13" t="s">
+      <c r="R2" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="S2" s="9" t="s">
+      <c r="S2" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="T2" s="9"/>
-      <c r="U2" s="9"/>
-      <c r="V2" s="9"/>
-      <c r="W2" s="9"/>
-      <c r="X2" s="9"/>
-      <c r="Y2" s="9"/>
-      <c r="Z2" s="9"/>
+      <c r="T2" s="13"/>
+      <c r="U2" s="13"/>
+      <c r="V2" s="13"/>
+      <c r="W2" s="13"/>
+      <c r="X2" s="13"/>
+      <c r="Y2" s="13"/>
+      <c r="Z2" s="13"/>
     </row>
     <row r="3" spans="1:26" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
-      <c r="C3" s="15"/>
+      <c r="C3" s="8"/>
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
       <c r="F3" s="8"/>
       <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="12"/>
-      <c r="O3" s="12"/>
-      <c r="P3" s="13"/>
-      <c r="Q3" s="13"/>
-      <c r="R3" s="13"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
       <c r="S3" s="3" t="s">
         <v>22</v>
       </c>
@@ -1555,24 +1571,20 @@
       <c r="Z3" s="3" t="s">
         <v>27</v>
       </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="V4" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="R2:R3"/>
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
-    <mergeCell ref="P2:P3"/>
-    <mergeCell ref="Q2:Q3"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="J1:O1"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="I1:O1"/>
     <mergeCell ref="P1:R1"/>
     <mergeCell ref="S1:Z1"/>
     <mergeCell ref="S2:Z2"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="E2:E3"/>
     <mergeCell ref="F2:F3"/>
@@ -1581,6 +1593,13 @@
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="K2:K3"/>
+    <mergeCell ref="R2:R3"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="Q2:Q3"/>
   </mergeCells>
   <dataValidations count="9">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Tình trạng sử dụng của công cụ dụng cụ: Còn sử dụng được và Không sử dụng được" sqref="N4:N2003" xr:uid="{D7D8503B-1533-4BDA-9D09-20E03F393295}">
@@ -1590,7 +1609,7 @@
       <formula1>1</formula1>
       <formula2>10000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Đơn giá ghi rõ giá trị của công cụ dụng cụ (mệnh giá: VNĐ)_x000a_Ví dụ: Đơn giá công cụ dụng cụ là 100,000 (Một trăm ngàn đồng) =&gt; Điền thông tin: 100000" sqref="K4:K2003" xr:uid="{E49CB6F3-5D33-4EC9-9F1E-5B9F4A14BF18}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Đơn giá ghi rõ giá trị của công cụ dụng cụ (mệnh giá: VNĐ)_x000a_Ví dụ: Đơn giá công cụ dụng cụ là 100,000 (Một trăm ngàn đồng) =&gt; Điền thông tin: 100000" sqref="J4:J2003" xr:uid="{E49CB6F3-5D33-4EC9-9F1E-5B9F4A14BF18}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Thể loại kỳ phân bổ tài sản công cụ dụng cụ: 1 lần, tháng, năm" sqref="P4:P2003" xr:uid="{93251718-4953-4151-9473-009C710C23B6}">
       <formula1>"1 lần,Tháng,Năm"</formula1>
     </dataValidation>
@@ -1600,7 +1619,7 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Số kỳ đã phân bổ tài sản công cụ dụng cụ" sqref="R4:R2003" xr:uid="{3E3AF060-E1B0-46C0-95B4-1A205C10B834}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Định dạng ngày sản xuất (dd/mm/yyyy)_x000a_Ví dụ: 10/10/2020" sqref="U4:U2003" xr:uid="{176D4A2E-5389-4EEB-9EC6-D07BBE5FE67D}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Định dạng hạn sử dụng (dd/mm/yyyy)_x000a_Ví dụ: 10/10/2024" sqref="V4:V2003" xr:uid="{A587C730-C6AC-4E9D-9AC3-AAD69DF64901}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Nhập số năm bắt đầu sử dụng của công cụ dụng cụ. Trường hợp không xác định được năm bắt đầu sử dụng điền &quot;N/A&quot;" sqref="G4:G2003" xr:uid="{1D7CE9E6-A1F7-4678-B810-8D650A343CEB}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Nhập số năm bắt đầu sử dụng của công cụ dụng cụ. Trường hợp không xác định được năm bắt đầu sử dụng điền &quot;N/A&quot;" sqref="F4:F2003" xr:uid="{1D7CE9E6-A1F7-4678-B810-8D650A343CEB}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update download file template import tool
</commit_message>
<xml_diff>
--- a/src/main/resources/static/Sample_Excel_Import_Tool.xlsx
+++ b/src/main/resources/static/Sample_Excel_Import_Tool.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hieux\Desktop\Projects\src\main\resources\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F4B9E5-FA6C-4A76-AB62-B973D400952E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E42B48-3042-4138-97B9-C622FEAD7B94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{69C10241-C50D-4A10-BA91-0773532975B3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{69C10241-C50D-4A10-BA91-0773532975B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Huongdannhapthongtin" sheetId="2" r:id="rId1"/>
@@ -429,12 +429,6 @@
     <t>Loại thiết bị y tế, dùng để xác định thông tin chi tiết về công cụ dụng cụ là thiết bị y tế</t>
   </si>
   <si>
-    <t>Ngày sản xuất thiết bị, dùng để xác định thông tin ngày sản xuất của công cụ dụng cụ</t>
-  </si>
-  <si>
-    <t>Hạn sử dụng, dùng để xác định ngày hết hạn của thiết bị</t>
-  </si>
-  <si>
     <t>Số lưu hành là số hiệu do đơn vị cung cấp quyết định khi lưu hành thiết bị.</t>
   </si>
   <si>
@@ -462,13 +456,63 @@
   <si>
     <t>Bao gồm các nhóm loại công cụ dụng cụ đã được xác định trong hệ thống. Người dùng sẽ chọn  công cụ dụng cụ đã được xác định từ danh sách công cụ dụng cụ.
 Người dùng có thể mở sheet "ToolCategoriesView" để xem danh sách danh mục công cụ dụng cụ tương ứng.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Ngày sản xuất thiết bị, dùng để xác định thông tin ngày sản xuất của công cụ dụng cụ
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Ví dụ:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 08/03/2024</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Hạn sử dụng, dùng để xác định ngày hết hạn của thiết bị
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Ví dụ:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 08/03/2024</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -512,6 +556,13 @@
     <font>
       <b/>
       <sz val="16"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -677,6 +728,28 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -686,25 +759,22 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -713,31 +783,12 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1104,126 +1155,126 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="10" t="s">
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
-      <c r="P1" s="11" t="s">
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="Q1" s="11"/>
-      <c r="R1" s="11"/>
-      <c r="S1" s="12" t="s">
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="T1" s="12"/>
-      <c r="U1" s="12"/>
-      <c r="V1" s="12"/>
-      <c r="W1" s="12"/>
-      <c r="X1" s="12"/>
-      <c r="Y1" s="12"/>
-      <c r="Z1" s="12"/>
+      <c r="T1" s="8"/>
+      <c r="U1" s="8"/>
+      <c r="V1" s="8"/>
+      <c r="W1" s="8"/>
+      <c r="X1" s="8"/>
+      <c r="Y1" s="8"/>
+      <c r="Z1" s="8"/>
     </row>
     <row r="2" spans="1:26" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="L2" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="M2" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="6" t="s">
+      <c r="N2" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="O2" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="P2" s="7" t="s">
+      <c r="P2" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="7" t="s">
+      <c r="Q2" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="R2" s="7" t="s">
+      <c r="R2" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="S2" s="13" t="s">
+      <c r="S2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="T2" s="13"/>
-      <c r="U2" s="13"/>
-      <c r="V2" s="13"/>
-      <c r="W2" s="13"/>
-      <c r="X2" s="13"/>
-      <c r="Y2" s="13"/>
-      <c r="Z2" s="13"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="10"/>
+      <c r="W2" s="10"/>
+      <c r="X2" s="10"/>
+      <c r="Y2" s="10"/>
+      <c r="Z2" s="10"/>
     </row>
     <row r="3" spans="1:26" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6"/>
-      <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
-      <c r="R3" s="7"/>
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="14"/>
+      <c r="N3" s="14"/>
+      <c r="O3" s="14"/>
+      <c r="P3" s="11"/>
+      <c r="Q3" s="11"/>
+      <c r="R3" s="11"/>
       <c r="S3" s="3" t="s">
         <v>22</v>
       </c>
@@ -1251,13 +1302,13 @@
     </row>
     <row r="4" spans="1:26" ht="179.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>32</v>
@@ -1272,7 +1323,7 @@
         <v>34</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>36</v>
@@ -1311,62 +1362,73 @@
         <v>23</v>
       </c>
       <c r="U4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="W4" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="V4" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="W4" s="2" t="s">
-        <v>49</v>
       </c>
       <c r="X4" s="2"/>
       <c r="Y4" s="2"/>
       <c r="Z4" s="2"/>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
+      <c r="A7" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
+      <c r="A9" s="13"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
+      <c r="A14" s="13"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A7:C14"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="L2:L3"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="I1:O1"/>
     <mergeCell ref="P1:R1"/>
@@ -1380,17 +1442,6 @@
     <mergeCell ref="S2:Z2"/>
     <mergeCell ref="Q2:Q3"/>
     <mergeCell ref="R2:R3"/>
-    <mergeCell ref="A7:C14"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
-    <mergeCell ref="P2:P3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="L2:L3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1427,126 +1478,126 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="19" t="s">
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="11" t="s">
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="20"/>
+      <c r="P1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="Q1" s="11"/>
-      <c r="R1" s="11"/>
-      <c r="S1" s="12" t="s">
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="T1" s="12"/>
-      <c r="U1" s="12"/>
-      <c r="V1" s="12"/>
-      <c r="W1" s="12"/>
-      <c r="X1" s="12"/>
-      <c r="Y1" s="12"/>
-      <c r="Z1" s="12"/>
+      <c r="T1" s="8"/>
+      <c r="U1" s="8"/>
+      <c r="V1" s="8"/>
+      <c r="W1" s="8"/>
+      <c r="X1" s="8"/>
+      <c r="Y1" s="8"/>
+      <c r="Z1" s="8"/>
     </row>
     <row r="2" spans="1:26" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="14" t="s">
+      <c r="H2" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="22" t="s">
+      <c r="K2" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="L2" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="M2" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="6" t="s">
+      <c r="N2" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="O2" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="P2" s="7" t="s">
+      <c r="P2" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="7" t="s">
+      <c r="Q2" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="R2" s="7" t="s">
+      <c r="R2" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="S2" s="13" t="s">
+      <c r="S2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="T2" s="13"/>
-      <c r="U2" s="13"/>
-      <c r="V2" s="13"/>
-      <c r="W2" s="13"/>
-      <c r="X2" s="13"/>
-      <c r="Y2" s="13"/>
-      <c r="Z2" s="13"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="10"/>
+      <c r="W2" s="10"/>
+      <c r="X2" s="10"/>
+      <c r="Y2" s="10"/>
+      <c r="Z2" s="10"/>
     </row>
     <row r="3" spans="1:26" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="23"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6"/>
-      <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
-      <c r="R3" s="7"/>
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="24"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="14"/>
+      <c r="N3" s="14"/>
+      <c r="O3" s="14"/>
+      <c r="P3" s="11"/>
+      <c r="Q3" s="11"/>
+      <c r="R3" s="11"/>
       <c r="S3" s="3" t="s">
         <v>22</v>
       </c>
@@ -1573,10 +1624,17 @@
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="V4" s="24"/>
+      <c r="V4" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="R2:R3"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="Q2:Q3"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="I1:O1"/>
     <mergeCell ref="P1:R1"/>
@@ -1593,13 +1651,6 @@
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="K2:K3"/>
-    <mergeCell ref="R2:R3"/>
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
-    <mergeCell ref="P2:P3"/>
-    <mergeCell ref="Q2:Q3"/>
   </mergeCells>
   <dataValidations count="9">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Tình trạng sử dụng của công cụ dụng cụ: Còn sử dụng được và Không sử dụng được" sqref="N4:N2003" xr:uid="{D7D8503B-1533-4BDA-9D09-20E03F393295}">

</xml_diff>

<commit_message>
create api upload file import tool
</commit_message>
<xml_diff>
--- a/src/main/resources/static/Sample_Excel_Import_Tool.xlsx
+++ b/src/main/resources/static/Sample_Excel_Import_Tool.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hieux\Desktop\Projects\src\main\resources\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E42B48-3042-4138-97B9-C622FEAD7B94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84724228-19CE-459F-8171-2ED8BD7BF156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{69C10241-C50D-4A10-BA91-0773532975B3}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{69C10241-C50D-4A10-BA91-0773532975B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Huongdannhapthongtin" sheetId="2" r:id="rId1"/>
@@ -729,6 +729,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -741,23 +756,8 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1155,40 +1155,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="6" t="s">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6"/>
-      <c r="N1" s="6"/>
-      <c r="O1" s="6"/>
-      <c r="P1" s="7" t="s">
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
-      <c r="S1" s="8" t="s">
+      <c r="Q1" s="12"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="T1" s="8"/>
-      <c r="U1" s="8"/>
-      <c r="V1" s="8"/>
-      <c r="W1" s="8"/>
-      <c r="X1" s="8"/>
-      <c r="Y1" s="8"/>
-      <c r="Z1" s="8"/>
+      <c r="T1" s="13"/>
+      <c r="U1" s="13"/>
+      <c r="V1" s="13"/>
+      <c r="W1" s="13"/>
+      <c r="X1" s="13"/>
+      <c r="Y1" s="13"/>
+      <c r="Z1" s="13"/>
     </row>
     <row r="2" spans="1:26" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
@@ -1215,46 +1215,46 @@
       <c r="H2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="I2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="14" t="s">
+      <c r="J2" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="14" t="s">
+      <c r="K2" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="14" t="s">
+      <c r="L2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="14" t="s">
+      <c r="M2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="14" t="s">
+      <c r="N2" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="14" t="s">
+      <c r="O2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="P2" s="11" t="s">
+      <c r="P2" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="11" t="s">
+      <c r="Q2" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="R2" s="11" t="s">
+      <c r="R2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="S2" s="10" t="s">
+      <c r="S2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="T2" s="10"/>
-      <c r="U2" s="10"/>
-      <c r="V2" s="10"/>
-      <c r="W2" s="10"/>
-      <c r="X2" s="10"/>
-      <c r="Y2" s="10"/>
-      <c r="Z2" s="10"/>
+      <c r="T2" s="14"/>
+      <c r="U2" s="14"/>
+      <c r="V2" s="14"/>
+      <c r="W2" s="14"/>
+      <c r="X2" s="14"/>
+      <c r="Y2" s="14"/>
+      <c r="Z2" s="14"/>
     </row>
     <row r="3" spans="1:26" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
@@ -1265,16 +1265,16 @@
       <c r="F3" s="9"/>
       <c r="G3" s="9"/>
       <c r="H3" s="9"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
-      <c r="P3" s="11"/>
-      <c r="Q3" s="11"/>
-      <c r="R3" s="11"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="8"/>
+      <c r="Q3" s="8"/>
+      <c r="R3" s="8"/>
       <c r="S3" s="3" t="s">
         <v>22</v>
       </c>
@@ -1375,60 +1375,49 @@
       <c r="Z4" s="2"/>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A8" s="13"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A9" s="13"/>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A10" s="13"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A11" s="13"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A12" s="13"/>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A13" s="13"/>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A14" s="13"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A7:C14"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
-    <mergeCell ref="P2:P3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="L2:L3"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="I1:O1"/>
     <mergeCell ref="P1:R1"/>
@@ -1442,6 +1431,17 @@
     <mergeCell ref="S2:Z2"/>
     <mergeCell ref="Q2:Q3"/>
     <mergeCell ref="R2:R3"/>
+    <mergeCell ref="A7:C14"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="L2:L3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1497,21 +1497,21 @@
       <c r="M1" s="19"/>
       <c r="N1" s="19"/>
       <c r="O1" s="20"/>
-      <c r="P1" s="7" t="s">
+      <c r="P1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
-      <c r="S1" s="8" t="s">
+      <c r="Q1" s="12"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="T1" s="8"/>
-      <c r="U1" s="8"/>
-      <c r="V1" s="8"/>
-      <c r="W1" s="8"/>
-      <c r="X1" s="8"/>
-      <c r="Y1" s="8"/>
-      <c r="Z1" s="8"/>
+      <c r="T1" s="13"/>
+      <c r="U1" s="13"/>
+      <c r="V1" s="13"/>
+      <c r="W1" s="13"/>
+      <c r="X1" s="13"/>
+      <c r="Y1" s="13"/>
+      <c r="Z1" s="13"/>
     </row>
     <row r="2" spans="1:26" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
@@ -1538,46 +1538,46 @@
       <c r="H2" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="I2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="14" t="s">
+      <c r="J2" s="7" t="s">
         <v>28</v>
       </c>
       <c r="K2" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="14" t="s">
+      <c r="L2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="14" t="s">
+      <c r="M2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="14" t="s">
+      <c r="N2" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="14" t="s">
+      <c r="O2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="P2" s="11" t="s">
+      <c r="P2" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="11" t="s">
+      <c r="Q2" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="R2" s="11" t="s">
+      <c r="R2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="S2" s="10" t="s">
+      <c r="S2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="T2" s="10"/>
-      <c r="U2" s="10"/>
-      <c r="V2" s="10"/>
-      <c r="W2" s="10"/>
-      <c r="X2" s="10"/>
-      <c r="Y2" s="10"/>
-      <c r="Z2" s="10"/>
+      <c r="T2" s="14"/>
+      <c r="U2" s="14"/>
+      <c r="V2" s="14"/>
+      <c r="W2" s="14"/>
+      <c r="X2" s="14"/>
+      <c r="Y2" s="14"/>
+      <c r="Z2" s="14"/>
     </row>
     <row r="3" spans="1:26" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
@@ -1588,16 +1588,16 @@
       <c r="F3" s="9"/>
       <c r="G3" s="9"/>
       <c r="H3" s="22"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
       <c r="K3" s="24"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
-      <c r="P3" s="11"/>
-      <c r="Q3" s="11"/>
-      <c r="R3" s="11"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="8"/>
+      <c r="Q3" s="8"/>
+      <c r="R3" s="8"/>
       <c r="S3" s="3" t="s">
         <v>22</v>
       </c>
@@ -1628,13 +1628,6 @@
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="R2:R3"/>
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
-    <mergeCell ref="P2:P3"/>
-    <mergeCell ref="Q2:Q3"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="I1:O1"/>
     <mergeCell ref="P1:R1"/>
@@ -1651,6 +1644,13 @@
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="K2:K3"/>
+    <mergeCell ref="R2:R3"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="Q2:Q3"/>
   </mergeCells>
   <dataValidations count="9">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Tình trạng sử dụng của công cụ dụng cụ: Còn sử dụng được và Không sử dụng được" sqref="N4:N2003" xr:uid="{D7D8503B-1533-4BDA-9D09-20E03F393295}">
@@ -1660,17 +1660,21 @@
       <formula1>1</formula1>
       <formula2>10000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Đơn giá ghi rõ giá trị của công cụ dụng cụ (mệnh giá: VNĐ)_x000a_Ví dụ: Đơn giá công cụ dụng cụ là 100,000 (Một trăm ngàn đồng) =&gt; Điền thông tin: 100000" sqref="J4:J2003" xr:uid="{E49CB6F3-5D33-4EC9-9F1E-5B9F4A14BF18}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Thể loại kỳ phân bổ tài sản công cụ dụng cụ: 1 lần, tháng, năm" sqref="P4:P2003" xr:uid="{93251718-4953-4151-9473-009C710C23B6}">
       <formula1>"1 lần,Tháng,Năm"</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Số kỳ phân bổ định dạng là số_x000a_Ví dụ: _x000a_1. Kỳ phân bổ là: Tháng_x000a_2. Số kỳ phân bổ: 24" sqref="Q4:Q2003" xr:uid="{42131C30-947C-4BE8-BEBD-3212A92C099F}">
-      <formula1>1</formula1>
-    </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Số kỳ đã phân bổ tài sản công cụ dụng cụ" sqref="R4:R2003" xr:uid="{3E3AF060-E1B0-46C0-95B4-1A205C10B834}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Định dạng ngày sản xuất (dd/mm/yyyy)_x000a_Ví dụ: 10/10/2020" sqref="U4:U2003" xr:uid="{176D4A2E-5389-4EEB-9EC6-D07BBE5FE67D}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Định dạng hạn sử dụng (dd/mm/yyyy)_x000a_Ví dụ: 10/10/2024" sqref="V4:V2003" xr:uid="{A587C730-C6AC-4E9D-9AC3-AAD69DF64901}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Nhập số năm bắt đầu sử dụng của công cụ dụng cụ. Trường hợp không xác định được năm bắt đầu sử dụng điền &quot;N/A&quot;" sqref="F4:F2003" xr:uid="{1D7CE9E6-A1F7-4678-B810-8D650A343CEB}"/>
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Đơn giá ghi rõ giá trị của công cụ dụng cụ (mệnh giá: VNĐ)_x000a_Ví dụ: Đơn giá công cụ dụng cụ là 100,000 (Một trăm ngàn đồng) =&gt; Điền thông tin: 100000" sqref="J4:J1048576" xr:uid="{8217F104-24B2-42BF-883C-D975BDBBF20F}">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Số kỳ phân bổ định dạng là số_x000a_Ví dụ: _x000a_1. Kỳ phân bổ là: Tháng_x000a_2. Số kỳ phân bổ: 24" sqref="Q4:Q1048576" xr:uid="{902A52C4-F004-4FA2-A540-41FCBFD459E4}">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Thông báo" prompt="Số kỳ đã phân bổ tài sản công cụ dụng cụ" sqref="R4:R1048576" xr:uid="{15998B25-ACC9-44EB-A2A5-273D912A515B}">
+      <formula1>0</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>